<commit_message>
score added for visualisation
</commit_message>
<xml_diff>
--- a/CW_Random_with_solution.xlsx
+++ b/CW_Random_with_solution.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,6 +422,11 @@
           <t>Result</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ProblemID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -450,6 +455,9 @@
 </t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -492,6 +500,9 @@
 </t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>232</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -540,6 +551,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B4" t="n">
+        <v>235</v>
       </c>
     </row>
     <row r="5">
@@ -579,6 +593,9 @@
 </t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>234</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -615,6 +632,9 @@
 </t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>236</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -646,6 +666,9 @@
 </t>
         </is>
       </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -682,6 +705,9 @@
 </t>
         </is>
       </c>
+      <c r="B8" t="n">
+        <v>233</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -706,6 +732,9 @@
 </t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -747,6 +776,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -784,6 +816,9 @@
 </t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -816,6 +851,9 @@
 </t>
         </is>
       </c>
+      <c r="B12" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -841,6 +879,9 @@
 </t>
         </is>
       </c>
+      <c r="B13" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -873,6 +914,9 @@
 </t>
         </is>
       </c>
+      <c r="B14" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -941,6 +985,9 @@
 </t>
         </is>
       </c>
+      <c r="B15" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -969,6 +1016,9 @@
 </t>
         </is>
       </c>
+      <c r="B16" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1001,6 +1051,9 @@
 </t>
         </is>
       </c>
+      <c r="B17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1029,6 +1082,9 @@
 </t>
         </is>
       </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1049,6 +1105,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B19" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="20">
@@ -1078,6 +1137,9 @@
 </t>
         </is>
       </c>
+      <c r="B20" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1101,6 +1163,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B21" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="22">
@@ -1118,6 +1183,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B22" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -1148,6 +1216,9 @@
 </t>
         </is>
       </c>
+      <c r="B23" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1182,6 +1253,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B24" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="25">
@@ -1229,6 +1303,9 @@
 </t>
         </is>
       </c>
+      <c r="B25" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1263,6 +1340,9 @@
 </t>
         </is>
       </c>
+      <c r="B26" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1284,6 +1364,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B27" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="28">
@@ -1330,6 +1413,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B28" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="29">
@@ -1352,6 +1438,9 @@
 </t>
         </is>
       </c>
+      <c r="B29" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1381,6 +1470,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B30" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="31">
@@ -1422,6 +1514,9 @@
 </t>
         </is>
       </c>
+      <c r="B31" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1434,6 +1529,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B32" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="33">
@@ -1462,6 +1560,9 @@
 </t>
         </is>
       </c>
+      <c r="B33" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1485,6 +1586,9 @@
 </t>
         </is>
       </c>
+      <c r="B34" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1509,6 +1613,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B35" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="36">
@@ -1548,6 +1655,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B36" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="37">
@@ -1584,6 +1694,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B37" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="38">
@@ -1612,6 +1725,9 @@
 </t>
         </is>
       </c>
+      <c r="B38" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1698,6 +1814,9 @@
 </t>
         </is>
       </c>
+      <c r="B39" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1730,6 +1849,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B40" t="n">
+        <v>107</v>
       </c>
     </row>
     <row r="41">
@@ -1753,6 +1875,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B41" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="42">
@@ -1801,6 +1926,9 @@
 </t>
         </is>
       </c>
+      <c r="B42" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1823,6 +1951,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B43" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="44">
@@ -1845,6 +1976,9 @@
 </t>
         </is>
       </c>
+      <c r="B44" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1873,6 +2007,9 @@
 </t>
         </is>
       </c>
+      <c r="B45" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1891,6 +2028,9 @@
 </t>
         </is>
       </c>
+      <c r="B46" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1923,6 +2063,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B47" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="48">
@@ -1991,6 +2134,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B48" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="49">
@@ -2017,6 +2163,9 @@
 </t>
         </is>
       </c>
+      <c r="B49" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2070,6 +2219,9 @@
 </t>
         </is>
       </c>
+      <c r="B50" t="n">
+        <v>112</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2101,6 +2253,9 @@
 }
 </t>
         </is>
+      </c>
+      <c r="B51" t="n">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>